<commit_message>
feat: master forms page + homepage revisions (Denis 21.06)
New: /master — tabbed preview of every form (accueil, inscription client/
fournisseur, connexion, 2350) accessible by direct link WITHOUT registering
(pure-CSS tabs, iframes; 2350 tab activates once a fiche is imported).

Homepage per Denis's notes:
- Promotion banner « avant le 1er sept 2026, aucun frais d'abonnement ».
- Launch date 1er août -> 1er octobre 2026.
- Suggestion line moved up, under the « recrutement perpétuel » phrase.
- Postal-code block moved under « 1er clic »; standalone search block removed;
  « en vert » now actually green.
- Removed the « 3e clic » lines (process is 2 clicks).
- Supplier « 6 options » now lists all 6 (was 5).
- Catalogue note all black; FOURNISSEURS/servclient line bigger.
- Removed the bottom CMS bloc (CIRKLE/Important/Suggestion) from the homepage.
- Tighter spacing (slideshow 240px, gaps 30px) — « moins d'espace ».

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/CIRKLE PAGE ACCUEIL 010626.xlsx
+++ b/docs/CIRKLE PAGE ACCUEIL 010626.xlsx
@@ -1125,191 +1125,6 @@
     <font>
       <b/>
       <i val="0"/>
-      <sz val="12"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <i val="0"/>
-      <sz val="12"/>
-      <color theme="9" tint="-0.25"/>
-      <name val="Calibri"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <i val="0"/>
-      <sz val="12"/>
-      <color theme="8" tint="-0.25"/>
-      <name val="Calibri"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <i val="0"/>
-      <sz val="14"/>
-      <color theme="9" tint="-0.25"/>
-      <name val="Calibri"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <i val="0"/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <i val="0"/>
-      <sz val="12"/>
-      <color auto="1"/>
-      <name val="Calibri"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <i val="0"/>
-      <sz val="11"/>
-      <color theme="5"/>
-      <name val="Calibri"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <i val="0"/>
-      <sz val="12"/>
-      <color rgb="FF00B050"/>
-      <name val="Calibri"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="0"/>
-      <i val="0"/>
-      <sz val="10"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <i val="0"/>
-      <sz val="10"/>
-      <color theme="9" tint="-0.25"/>
-      <name val="Calibri"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <i val="0"/>
-      <sz val="12"/>
-      <color rgb="FF00B050"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <b/>
-      <i val="0"/>
-      <sz val="12"/>
-      <color rgb="FF2F75B5"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <b/>
-      <i val="0"/>
-      <sz val="11"/>
-      <color rgb="FF00B050"/>
-      <name val="Calibri"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <i val="0"/>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <b val="0"/>
-      <i val="0"/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <b/>
-      <i val="0"/>
-      <sz val="11"/>
-      <color theme="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <b val="0"/>
-      <i val="0"/>
-      <sz val="12"/>
-      <color rgb="FF0070C0"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <b/>
-      <i val="0"/>
-      <sz val="12"/>
-      <color rgb="FF0070C0"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <b/>
-      <i val="0"/>
-      <sz val="12"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <i val="0"/>
-      <sz val="11"/>
-      <color theme="10"/>
-      <name val="Calibri"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <i val="0"/>
-      <sz val="12"/>
-      <color theme="0" tint="-0.35"/>
-      <name val="Calibri"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <i val="0"/>
-      <sz val="14"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <i val="0"/>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <i val="0"/>
-      <sz val="14"/>
-      <color rgb="FF0070C0"/>
-      <name val="Calibri"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <i val="0"/>
       <sz val="11"/>
       <color rgb="FF0070C0"/>
       <name val="Arial"/>
@@ -1317,16 +1132,7 @@
     <font>
       <b/>
       <i val="0"/>
-      <u/>
-      <sz val="16"/>
-      <color theme="10"/>
-      <name val="Calibri"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <i val="0"/>
-      <sz val="12"/>
+      <sz val="11"/>
       <color rgb="FFFF0000"/>
       <name val="Arial"/>
     </font>
@@ -1347,11 +1153,156 @@
       <name val="Arial"/>
     </font>
     <font>
+      <b val="0"/>
+      <i val="0"/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <i val="0"/>
+      <sz val="12"/>
+      <color rgb="FFFF0000"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <i val="0"/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <i val="0"/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <b val="0"/>
+      <i val="0"/>
+      <sz val="12"/>
+      <color rgb="FF0070C0"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <i val="0"/>
+      <u/>
+      <sz val="16"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <i val="0"/>
+      <sz val="12"/>
+      <color rgb="FF0070C0"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <i val="0"/>
+      <sz val="12"/>
+      <color rgb="FF00B050"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <i val="0"/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <i val="0"/>
+      <sz val="12"/>
+      <color rgb="FF00B050"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <i val="0"/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <i val="0"/>
+      <sz val="12"/>
+      <color rgb="FF2F75B5"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <i val="0"/>
+      <sz val="14"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <i val="0"/>
+      <sz val="12"/>
+      <color auto="1"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="0"/>
+      <i val="0"/>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <i val="0"/>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <i val="0"/>
+      <sz val="12"/>
+      <color theme="0" tint="-0.35"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <i val="0"/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <b/>
       <i val="0"/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <i val="0"/>
+      <sz val="14"/>
+      <color rgb="FF0070C0"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <b val="0"/>
@@ -1364,8 +1315,40 @@
     <font>
       <b/>
       <i val="0"/>
+      <sz val="14"/>
+      <color theme="9" tint="-0.25"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <i val="0"/>
       <sz val="12"/>
       <color rgb="FF0070C0"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <i val="0"/>
+      <sz val="12"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <i val="0"/>
+      <sz val="12"/>
+      <color theme="9" tint="-0.25"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <i val="0"/>
+      <sz val="10"/>
+      <color theme="9" tint="-0.25"/>
       <name val="Calibri"/>
       <scheme val="minor"/>
     </font>
@@ -1389,8 +1372,25 @@
       <b/>
       <i val="0"/>
       <sz val="12"/>
-      <color theme="1"/>
-      <name val="Arial"/>
+      <color theme="8" tint="-0.25"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <i val="0"/>
+      <sz val="11"/>
+      <color rgb="FF00B050"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <i val="0"/>
+      <sz val="11"/>
+      <color theme="5"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="5">
@@ -1402,12 +1402,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
+        <fgColor theme="7" tint="0.6"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.6"/>
+        <fgColor rgb="FFFFFF00"/>
       </patternFill>
     </fill>
     <fill>
@@ -1434,9 +1434,36 @@
       <diagonal/>
     </border>
     <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left style="medium">
         <color rgb="FF000000"/>
       </left>
+      <right/>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
       <right style="medium">
         <color rgb="FF000000"/>
       </right>
@@ -1450,10 +1477,64 @@
       <left style="medium">
         <color rgb="FF000000"/>
       </left>
+      <right/>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
       <right style="medium">
         <color rgb="FF000000"/>
       </right>
-      <top/>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
       <bottom/>
       <diagonal/>
     </border>
@@ -1461,24 +1542,6 @@
       <left style="medium">
         <color rgb="FF000000"/>
       </left>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FF000000"/>
-      </left>
       <right style="medium">
         <color rgb="FF000000"/>
       </right>
@@ -1492,13 +1555,57 @@
       <left style="medium">
         <color rgb="FF000000"/>
       </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
       <right style="medium">
         <color rgb="FF000000"/>
       </right>
-      <top style="medium">
+      <top/>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top style="thin">
         <color rgb="FF000000"/>
       </top>
-      <bottom style="medium">
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
         <color rgb="FF000000"/>
       </bottom>
       <diagonal/>
@@ -1537,6 +1644,17 @@
       </left>
       <right/>
       <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
       <bottom style="medium">
         <color rgb="FF000000"/>
       </bottom>
@@ -1545,47 +1663,6 @@
     <border>
       <left/>
       <right/>
-      <top/>
-      <bottom style="medium">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
       <top style="thin">
         <color rgb="FF000000"/>
       </top>
@@ -1599,7 +1676,9 @@
       <right style="medium">
         <color rgb="FF000000"/>
       </right>
-      <top/>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
       <bottom style="medium">
         <color rgb="FF000000"/>
       </bottom>
@@ -1608,6 +1687,15 @@
     <border>
       <left/>
       <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
         <color rgb="FF000000"/>
       </right>
       <top/>
@@ -1618,73 +1706,7 @@
       <left style="medium">
         <color rgb="FF000000"/>
       </left>
-      <right/>
-      <top style="medium">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="medium">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
       <right style="medium">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="medium">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FF000000"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
         <color rgb="FF000000"/>
       </right>
       <top/>
@@ -1692,77 +1714,27 @@
       <diagonal/>
     </border>
     <border>
-      <left style="medium">
+      <left style="thin">
         <color rgb="FF000000"/>
       </left>
-      <right/>
-      <top style="medium">
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
         <color rgb="FF000000"/>
       </top>
-      <bottom style="medium">
+      <bottom style="thin">
         <color rgb="FF000000"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
-      <top style="medium">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="medium">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
+      <left style="thin">
         <color rgb="FF000000"/>
       </left>
       <right/>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FF000000"/>
-      </bottom>
+      <top/>
+      <bottom/>
       <diagonal/>
     </border>
     <border>
@@ -1785,369 +1757,398 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="3">
+  <cellStyleXfs count="4">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyFill="0" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="131">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0">
-      <alignment horizontal="center" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0">
-      <alignment horizontal="center" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="2"/>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="2"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0">
+      <alignment horizontal="center" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0">
+      <alignment horizontal="center" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="3"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="3"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="3">
+      <alignment horizontal="center" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="3"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="3">
+      <alignment horizontal="center" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment horizontal="center" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0">
+      <alignment horizontal="center" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="3">
+      <alignment horizontal="center" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="3">
+      <alignment horizontal="center" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="3"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="3">
+      <alignment horizontal="center" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="3">
+      <alignment horizontal="center" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="4" xfId="3">
+      <alignment horizontal="center" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="5" xfId="3">
+      <alignment horizontal="center" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="6" xfId="3">
+      <alignment horizontal="center" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" xfId="3">
+      <alignment horizontal="center" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" xfId="3">
+      <alignment horizontal="center" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="2" xfId="3">
+      <alignment horizontal="center" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="9" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="3" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="4" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="5" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="10" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="11" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="12" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="2" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="13" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0">
+      <alignment horizontal="center" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="11" xfId="0">
+      <alignment horizontal="center" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="11" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="14" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="15" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="16" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="3" xfId="0">
+      <alignment horizontal="center" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="4" xfId="0">
+      <alignment horizontal="center" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="2">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="14" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="15" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="16" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="12" xfId="0">
+      <alignment horizontal="center" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="2" xfId="0">
+      <alignment horizontal="center" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="2">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="11" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="4"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="19" xfId="0">
+      <alignment horizontal="center" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0">
+      <alignment horizontal="center" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="19" xfId="0"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="2">
-      <alignment horizontal="center" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="2"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="2">
-      <alignment horizontal="center" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment horizontal="center" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="3" borderId="0" xfId="0">
-      <alignment horizontal="center" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="0" xfId="2">
-      <alignment horizontal="center" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="2">
-      <alignment horizontal="center" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="11" xfId="2"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="11" xfId="2">
-      <alignment horizontal="center" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="17" xfId="2">
-      <alignment horizontal="center" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="18" xfId="2">
-      <alignment horizontal="center" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="19" xfId="2">
-      <alignment horizontal="center" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="19" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="19" xfId="0">
+      <alignment horizontal="left" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0">
+      <alignment horizontal="left" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="9" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="4"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="20" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="24" xfId="2">
-      <alignment horizontal="center" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="25" xfId="2">
-      <alignment horizontal="center" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="26" xfId="2">
-      <alignment horizontal="center" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="11" xfId="2">
-      <alignment horizontal="center" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" xfId="0">
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="21" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="22" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="6" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="17" xfId="0">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="7" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="18" xfId="0">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="8" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="19" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="6" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="10" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="15" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0">
-      <alignment horizontal="center" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="0">
-      <alignment horizontal="center" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="6" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="20" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="21" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="22" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="17" xfId="0">
-      <alignment horizontal="center" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="18" xfId="0">
-      <alignment horizontal="center" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="20" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="21" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="22" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="10" xfId="0">
-      <alignment horizontal="center" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="11" xfId="0">
-      <alignment horizontal="center" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="6" xfId="0">
-      <alignment horizontal="left" vertical="center" indent="4"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="4" xfId="0">
-      <alignment horizontal="center" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" xfId="0">
-      <alignment horizontal="center" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0">
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="19" xfId="0">
       <alignment horizontal="left" vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0">
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="23" xfId="0">
       <alignment horizontal="left" vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" xfId="0">
-      <alignment horizontal="left" vertical="center" indent="4"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="27" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="28" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="29" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="24" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="25" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="26" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="4" xfId="0">
+    <xf numFmtId="0" fontId="26" fillId="3" borderId="12" xfId="0">
+      <alignment horizontal="center" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="3" borderId="2" xfId="0">
+      <alignment horizontal="center" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="3" borderId="13" xfId="0">
+      <alignment horizontal="center" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0">
+      <alignment horizontal="center" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0">
       <alignment horizontal="left" vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="16" xfId="0">
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="23" xfId="0">
       <alignment horizontal="left" vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="2" borderId="10" xfId="0">
-      <alignment horizontal="center" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="2" borderId="11" xfId="0">
-      <alignment horizontal="center" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="2" borderId="15" xfId="0">
-      <alignment horizontal="center" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0">
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0">
+      <alignment horizontal="left" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="23" xfId="0">
+      <alignment horizontal="left" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0">
+      <alignment horizontal="center" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="23" xfId="0">
+      <alignment horizontal="center" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0">
+      <alignment horizontal="center" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="2">
+      <alignment horizontal="left" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" xfId="0">
+      <alignment horizontal="center" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="23" xfId="0">
+      <alignment horizontal="center" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="2">
       <alignment horizontal="center" vertical="bottom"/>
     </xf>
     <xf numFmtId="0" fontId="34" fillId="0" borderId="0" xfId="0">
       <alignment horizontal="left" vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="16" xfId="0">
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="23" xfId="0">
       <alignment horizontal="left" vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0">
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0">
+      <alignment horizontal="center" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="24" xfId="0">
+      <alignment horizontal="center" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="25" xfId="0"/>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="23" xfId="0">
+      <alignment horizontal="center" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="26" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="19" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0">
+      <alignment horizontal="center" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0">
+      <alignment horizontal="center" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0">
+      <alignment horizontal="center" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="10" xfId="0">
+      <alignment horizontal="center" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="28" xfId="0">
+      <alignment horizontal="center" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="29" xfId="0">
+      <alignment horizontal="center" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0">
+      <alignment horizontal="center" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="19" xfId="0">
+      <alignment horizontal="center" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="26" xfId="0">
+      <alignment horizontal="center" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="0" xfId="0">
+      <alignment horizontal="center" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="19" xfId="0">
+      <alignment horizontal="center" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0">
+      <alignment horizontal="center" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0">
+      <alignment horizontal="center" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0">
+      <alignment horizontal="center" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0">
+      <alignment horizontal="center" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="19" xfId="0">
+      <alignment horizontal="center" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0">
+      <alignment horizontal="center" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="19" xfId="0">
+      <alignment horizontal="center" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="0" xfId="0">
+      <alignment horizontal="center" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="9" xfId="0">
+      <alignment horizontal="center" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="10" xfId="0">
+      <alignment horizontal="center" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="3" xfId="0">
+      <alignment horizontal="center" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="5" xfId="0">
+      <alignment horizontal="center" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0">
+      <alignment horizontal="center" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="25" xfId="0">
+      <alignment horizontal="center" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="23" xfId="0">
+      <alignment horizontal="center" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0">
+      <alignment horizontal="center" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="0" xfId="0">
       <alignment horizontal="left" vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="16" xfId="0">
-      <alignment horizontal="left" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0">
-      <alignment horizontal="center" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="16" xfId="0">
-      <alignment horizontal="center" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0">
-      <alignment horizontal="center" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="1">
-      <alignment horizontal="left" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="0" xfId="0">
-      <alignment horizontal="center" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="16" xfId="0">
-      <alignment horizontal="center" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="1">
-      <alignment horizontal="center" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="0" xfId="0">
-      <alignment horizontal="left" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="16" xfId="0">
-      <alignment horizontal="left" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0">
-      <alignment horizontal="center" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="23" xfId="0">
-      <alignment horizontal="center" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0"/>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="16" xfId="0">
-      <alignment horizontal="center" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="12" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="4" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0">
-      <alignment horizontal="center" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0">
-      <alignment horizontal="center" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0">
-      <alignment horizontal="center" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0">
-      <alignment horizontal="center" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="30" xfId="0">
-      <alignment horizontal="center" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="31" xfId="0">
-      <alignment horizontal="center" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0">
-      <alignment horizontal="center" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="4" xfId="0">
-      <alignment horizontal="center" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="12" xfId="0">
-      <alignment horizontal="center" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0">
-      <alignment horizontal="center" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0">
-      <alignment horizontal="center" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0">
-      <alignment horizontal="center" vertical="bottom"/>
-    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="25" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0">
-      <alignment horizontal="center" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0">
-      <alignment horizontal="center" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0">
-      <alignment horizontal="center" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0">
-      <alignment horizontal="center" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0">
-      <alignment horizontal="center" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0">
-      <alignment horizontal="center" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0">
-      <alignment horizontal="center" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0">
-      <alignment horizontal="center" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0">
-      <alignment horizontal="center" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0">
-      <alignment horizontal="center" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="19" xfId="0">
-      <alignment horizontal="center" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0">
-      <alignment horizontal="center" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0">
-      <alignment horizontal="center" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="16" xfId="0">
-      <alignment horizontal="center" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0">
-      <alignment horizontal="center" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0">
-      <alignment horizontal="left" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0">
       <alignment horizontal="center" vertical="bottom"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
-    <cellStyle name="Normal" xfId="0"/>
-    <cellStyle name="Heading 2" xfId="1" builtinId="17"/>
-    <cellStyle name="Hyperlink" xfId="2" builtinId="8"/>
+    <cellStyle name="Normal" xfId="1"/>
+    <cellStyle name="Heading 2" xfId="2" builtinId="17"/>
+    <cellStyle name="Hyperlink" xfId="3" builtinId="8"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -2747,7 +2748,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{6F5150A9-B462-405A-9C67-700B81614D1C}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{D63DAAED-89F9-46D3-AD05-002CDB42E99F}" mc:Ignorable="x14ac xr xr2 xr3">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
@@ -2799,7 +2800,7 @@
       <c r="F3" s="4"/>
       <c r="G3" s="4"/>
     </row>
-    <row r="4" ht="14.497499999999997" customHeight="1">
+    <row r="4" ht="14.25" customHeight="1">
       <c r="A4" s="5"/>
       <c r="B4" s="5"/>
       <c r="C4" s="5"/>
@@ -2819,7 +2820,7 @@
       <c r="F5" s="6"/>
       <c r="G5" s="6"/>
     </row>
-    <row r="6" ht="14.497499999999997" customHeight="1">
+    <row r="6" ht="14.25" customHeight="1">
       <c r="A6" s="5"/>
       <c r="B6" s="7"/>
       <c r="C6" s="7"/>
@@ -2856,7 +2857,7 @@
       <c r="M7" s="9"/>
       <c r="N7" s="9"/>
     </row>
-    <row r="8" ht="14.497499999999997" customHeight="1">
+    <row r="8" ht="14.25" customHeight="1">
       <c r="A8" s="5"/>
       <c r="B8" s="7"/>
       <c r="C8" s="7"/>
@@ -2867,7 +2868,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="9" ht="14.497499999999997" customHeight="1">
+    <row r="9" ht="14.25" customHeight="1">
       <c r="A9" s="5"/>
       <c r="B9" s="7"/>
       <c r="C9" s="7"/>
@@ -3563,7 +3564,7 @@
       <c r="E55" s="115"/>
       <c r="F55" s="103"/>
     </row>
-    <row r="56" ht="14.497499999999997" customHeight="1">
+    <row r="56" ht="14.25" customHeight="1">
       <c r="A56" s="117" t="s">
         <v>81</v>
       </c>
@@ -3585,7 +3586,7 @@
       <c r="E57" s="113"/>
       <c r="F57" s="113"/>
     </row>
-    <row r="58" ht="14.497499999999997" customHeight="1">
+    <row r="58" ht="14.25" customHeight="1">
       <c r="A58" s="121"/>
       <c r="B58" s="123"/>
       <c r="C58" s="124"/>
@@ -3593,14 +3594,14 @@
       <c r="E58" s="126"/>
       <c r="F58" s="126"/>
     </row>
-    <row r="59" ht="14.497499999999997" customHeight="1">
+    <row r="59" ht="14.25" customHeight="1">
       <c r="A59" s="121"/>
       <c r="B59" s="123"/>
       <c r="C59" s="124"/>
       <c r="D59" s="125"/>
       <c r="E59" s="9"/>
     </row>
-    <row r="60" ht="14.497499999999997" customHeight="1">
+    <row r="60" ht="14.25" customHeight="1">
       <c r="A60" s="125"/>
       <c r="B60" s="123"/>
       <c r="C60" s="124"/>
@@ -3608,7 +3609,7 @@
       <c r="E60" s="9"/>
       <c r="F60" s="9"/>
     </row>
-    <row r="61" ht="14.497499999999997" customHeight="1">
+    <row r="61" ht="14.25" customHeight="1">
       <c r="A61" s="121"/>
       <c r="B61" s="123"/>
       <c r="C61" s="124"/>
@@ -3616,7 +3617,7 @@
       <c r="E61" s="9"/>
       <c r="F61" s="9"/>
     </row>
-    <row r="62" ht="14.497499999999997" customHeight="1">
+    <row r="62" ht="14.25" customHeight="1">
       <c r="A62" s="127"/>
       <c r="B62" s="123"/>
       <c r="C62" s="124"/>
@@ -3700,6 +3701,12 @@
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="A3:G3" r:id="rId1" display=" SERVCLIENT@CIRKLESERVICES.COM"/>
+    <hyperlink ref="B3" r:id="rId2"/>
+    <hyperlink ref="C3" r:id="rId3"/>
+    <hyperlink ref="D3" r:id="rId4"/>
+    <hyperlink ref="E3" r:id="rId5"/>
+    <hyperlink ref="F3" r:id="rId6"/>
+    <hyperlink ref="G3" r:id="rId7"/>
   </hyperlinks>
   <printOptions/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3708,7 +3715,7 @@
     <oddHeader>&amp;L&amp;C&amp;R</oddHeader>
     <oddFooter>&amp;L&amp;C&amp;R</oddFooter>
   </headerFooter>
-  <drawing r:id="rId2"/>
+  <drawing r:id="rId8"/>
   <extLst/>
 </worksheet>
 </file>
</xml_diff>